<commit_message>
fix: clear hash-based computed id formulas for kind/publisher/provenance_statement/purpose too
The first commit on this branch only cleared computed/visible for the 6 tables newly
made independent here, on the assumption that kind/publisher/provenance_statement/
purpose - already fixed in Python code by PR #47/#57 - had their schema side handled
elsewhere too. They hadn't: their id columns still had the old server-computed hash
formula, so MOLGENIS was still silently overriding the UUID the harvester sends,
reproducing the exact same foreign-key violation live:

  Upsert into table 'collections' failed: ... foreign key (ref_array) constraint.
  Details: Key ("contactPoint")=(801c1651-...) is not present in table "kind",
  column(s)("id")

Clear computed/visible for these four tables' id column too, matching what's now
already done for the other six.
</commit_message>
<xml_diff>
--- a/dev/molgenis/D5.3 - EUCAIM - Molgenis metadata model - september 2026.xlsx
+++ b/dev/molgenis/D5.3 - EUCAIM - Molgenis metadata model - september 2026.xlsx
@@ -1201,14 +1201,6 @@
       <c r="G24" t="b">
         <v>1</v>
       </c>
-      <c r="O24" t="b">
-        <v>0</v>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>String([…name].sort().join('\0').split('').reduce((h, c) =&gt; Math.imul(h, 33) ^ c.charCodeAt(0), 5381) &gt;&gt;&gt; 0)</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4145,14 +4137,6 @@
       <c r="G109" t="b">
         <v>1</v>
       </c>
-      <c r="O109" t="b">
-        <v>0</v>
-      </c>
-      <c r="P109" t="inlineStr">
-        <is>
-          <t>fn.replaceAll(' ', '').toLowerCase()</t>
-        </is>
-      </c>
       <c r="Q109" s="4" t="n"/>
     </row>
     <row r="110">
@@ -5550,14 +5534,7 @@
       <c r="G153" t="b">
         <v>1</v>
       </c>
-      <c r="O153" t="b">
-        <v>0</v>
-      </c>
-      <c r="P153" s="15" t="inlineStr">
-        <is>
-          <t>String([...label].sort().join('\0').split('').reduce((h, c) =&gt; Math.imul(h, 33) ^ c.charCodeAt(0), 5381) &gt;&gt;&gt; 0)</t>
-        </is>
-      </c>
+      <c r="P153" s="15" t="n"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5611,14 +5588,7 @@
       <c r="G155" t="b">
         <v>1</v>
       </c>
-      <c r="O155" t="b">
-        <v>0</v>
-      </c>
-      <c r="P155" s="15" t="inlineStr">
-        <is>
-          <t>String([...description].sort().join('\0').split('').reduce((h, c) =&gt; Math.imul(h, 33) ^ c.charCodeAt(0), 5381) &gt;&gt;&gt; 0)</t>
-        </is>
-      </c>
+      <c r="P155" s="15" t="n"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">

</xml_diff>